<commit_message>
Update decay records for 34Cl and 34S with revised branching ratios, intensity details, and clarifications
</commit_message>
<xml_diff>
--- a/A34/Cl34/raw/34Clm_146isomer.xlsx
+++ b/A34/Cl34/raw/34Clm_146isomer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sun\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A34\Cl34\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551073A0-6955-488A-8E1F-E64AD0D646C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9FB1A2D-1EA9-4055-89ED-FA329C10806F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8736" yWindow="-60" windowWidth="12984" windowHeight="12396" xr2:uid="{64E99CE1-442C-4A7F-8B3B-37F466BBE269}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{64E99CE1-442C-4A7F-8B3B-37F466BBE269}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="13">
   <si>
     <t>34Clm</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>Evaluated</t>
+  </si>
+  <si>
+    <t>Red numbers are measured</t>
   </si>
 </sst>
 </file>
@@ -86,7 +89,7 @@
     <numFmt numFmtId="167" formatCode="0.00000"/>
     <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,6 +107,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -154,7 +165,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -238,6 +249,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -562,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F7FD4E-9B9E-4B69-B722-057952471005}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" style="1" bestFit="1" customWidth="1"/>
@@ -582,120 +596,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22" t="s">
-        <v>7</v>
+      <c r="A1" s="29" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3">
-        <v>129.30000000000001</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1.2</v>
-      </c>
-      <c r="D2" s="4">
-        <f>B2/B7</f>
-        <v>0.5546023848331475</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="5">
-        <f>D2/B2</f>
-        <v>4.2892682508364069E-3</v>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="I2" s="23">
-        <v>129.30000000000001</v>
-      </c>
-      <c r="J2" s="22">
-        <v>1.2</v>
-      </c>
-      <c r="K2" s="24">
-        <f>I2/I7</f>
-        <v>0.54025226145501926</v>
-      </c>
-      <c r="L2" s="24">
-        <v>4.4000000000000003E-3</v>
-      </c>
-      <c r="M2" s="25">
-        <f>K2/I2</f>
-        <v>4.1782850847255932E-3</v>
+        <v>0</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>94.4</v>
+        <v>129.30000000000001</v>
       </c>
       <c r="C3" s="2">
-        <v>1.4</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>1.2</v>
+      </c>
+      <c r="D3" s="4">
+        <f>B3/B8</f>
+        <v>0.5546023848331475</v>
+      </c>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="F3" s="5">
+        <f>D3/B3</f>
+        <v>4.2892682508364069E-3</v>
+      </c>
       <c r="H3" s="22" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="23">
-        <v>94.4</v>
+        <v>129.30000000000001</v>
       </c>
       <c r="J3" s="22">
-        <v>1.4</v>
-      </c>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
+        <v>1.2</v>
+      </c>
+      <c r="K3" s="24">
+        <f>I3/I8</f>
+        <v>0.54025226145501926</v>
+      </c>
+      <c r="L3" s="24">
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="M3" s="25">
+        <f>K3/I3</f>
+        <v>4.1782850847255932E-3</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="6">
-        <v>0.1</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
+        <v>94.4</v>
       </c>
       <c r="C4" s="2">
-        <v>8.9999999999999993E-3</v>
+        <v>1.4</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="H4" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" s="26">
-        <v>0.1656</v>
+        <v>2</v>
+      </c>
+      <c r="I4" s="23">
+        <v>94.4</v>
       </c>
       <c r="J4" s="22">
-        <v>2.3999999999999998E-3</v>
+        <v>1.4</v>
       </c>
       <c r="K4" s="22"/>
       <c r="L4" s="22"/>
@@ -703,25 +696,25 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2">
-        <f>B3*B4</f>
-        <v>9.4400000000000013</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="B5" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>8.9999999999999993E-3</v>
+      </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="H5" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="27">
-        <f>I3*I4</f>
-        <v>15.63264</v>
+        <v>6</v>
+      </c>
+      <c r="I5" s="26">
+        <v>0.1656</v>
       </c>
       <c r="J5" s="22">
-        <v>0.32</v>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="K5" s="22"/>
       <c r="L5" s="22"/>
@@ -729,120 +722,132 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7">
-        <f>B3+B5</f>
-        <v>103.84</v>
+        <v>3</v>
+      </c>
+      <c r="B6" s="2">
+        <f>B4*B5</f>
+        <v>9.4400000000000013</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="4">
-        <f>B6/B7</f>
-        <v>0.4453976151668525</v>
-      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="H6" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="I6" s="28">
-        <f>I3+I5</f>
-        <v>110.03264</v>
+        <v>3</v>
+      </c>
+      <c r="I6" s="27">
+        <f>I4*I5</f>
+        <v>15.63264</v>
       </c>
       <c r="J6" s="22">
-        <v>1.65</v>
-      </c>
-      <c r="K6" s="24">
-        <f>I6/I7</f>
-        <v>0.45974773854498069</v>
-      </c>
-      <c r="L6" s="24">
-        <v>4.4000000000000003E-3</v>
-      </c>
+        <v>0.32</v>
+      </c>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
       <c r="M6" s="22"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2">
-        <f>B2+B6</f>
-        <v>233.14000000000001</v>
+        <v>4</v>
+      </c>
+      <c r="B7" s="7">
+        <f>B4+B6</f>
+        <v>103.84</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="D7" s="4">
+        <f>B7/B8</f>
+        <v>0.4453976151668525</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="H7" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="28">
+        <f>I4+I6</f>
+        <v>110.03264</v>
+      </c>
+      <c r="J7" s="28">
+        <v>1.65</v>
+      </c>
+      <c r="K7" s="24">
+        <f>I7/I8</f>
+        <v>0.45974773854498069</v>
+      </c>
+      <c r="L7" s="24">
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="M7" s="22"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I7" s="27">
-        <f>I2+I6</f>
+      <c r="B8" s="2">
+        <f>B3+B7</f>
+        <v>233.14000000000001</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="H8" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="27">
+        <f>I3+I7</f>
         <v>239.33264000000003</v>
       </c>
-      <c r="J7" s="22">
+      <c r="J8" s="22">
         <v>2.04</v>
       </c>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B11" s="16">
         <f>100+25.4+0.52</f>
         <v>125.92</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C11" s="15">
         <v>1.2</v>
       </c>
-      <c r="D10" s="17">
-        <f>B10/B15</f>
+      <c r="D11" s="17">
+        <f>B11/B16</f>
         <v>0.53126318454138899</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="18">
-        <f>D10/B10</f>
+      <c r="E11" s="15"/>
+      <c r="F11" s="18">
+        <f>D11/B11</f>
         <v>4.2190532444519452E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" s="19">
-        <v>101</v>
-      </c>
-      <c r="C11" s="20">
-        <v>4</v>
-      </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="21">
-        <v>0.1</v>
-      </c>
-      <c r="C12" s="15">
-        <v>8.9999999999999993E-3</v>
+        <v>2</v>
+      </c>
+      <c r="B12" s="19">
+        <v>101</v>
+      </c>
+      <c r="C12" s="20">
+        <v>4</v>
       </c>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
@@ -850,104 +855,104 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="15">
-        <f>B11*B12</f>
-        <v>10.100000000000001</v>
-      </c>
-      <c r="C13" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="B13" s="21">
+        <v>0.1</v>
+      </c>
+      <c r="C13" s="15">
+        <v>8.9999999999999993E-3</v>
+      </c>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="20">
-        <f>B11+B13</f>
-        <v>111.1</v>
+        <v>3</v>
+      </c>
+      <c r="B14" s="15">
+        <f>B12*B13</f>
+        <v>10.100000000000001</v>
       </c>
       <c r="C14" s="15"/>
-      <c r="D14" s="17">
-        <f>B14/B15</f>
-        <v>0.46873681545861112</v>
-      </c>
+      <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="15">
-        <f>B10+B14</f>
-        <v>237.01999999999998</v>
+        <v>4</v>
+      </c>
+      <c r="B15" s="20">
+        <f>B12+B14</f>
+        <v>111.1</v>
       </c>
       <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
+      <c r="D15" s="17">
+        <f>B15/B16</f>
+        <v>0.46873681545861112</v>
+      </c>
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="15">
+        <f>B11+B15</f>
+        <v>237.01999999999998</v>
+      </c>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B19" s="9">
         <f>100+27.3+0.61</f>
         <v>127.91</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C19" s="8">
         <v>1.2</v>
       </c>
-      <c r="D18" s="10">
-        <f>B18/B23</f>
+      <c r="D19" s="10">
+        <f>B19/B24</f>
         <v>0.5488050800188784</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="11">
-        <f>D18/B18</f>
+      <c r="E19" s="8"/>
+      <c r="F19" s="11">
+        <f>D19/B19</f>
         <v>4.2905564851761268E-3</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" s="12">
-        <v>95.6</v>
-      </c>
-      <c r="C19" s="8">
-        <v>1.9</v>
-      </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="13">
-        <v>0.1</v>
+        <v>2</v>
+      </c>
+      <c r="B20" s="12">
+        <v>95.6</v>
       </c>
       <c r="C20" s="8">
-        <v>8.9999999999999993E-3</v>
+        <v>1.9</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
@@ -955,45 +960,59 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="8">
-        <f>B19*B20</f>
-        <v>9.56</v>
-      </c>
-      <c r="C21" s="8"/>
+        <v>6</v>
+      </c>
+      <c r="B21" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="C21" s="8">
+        <v>8.9999999999999993E-3</v>
+      </c>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="14">
-        <f>B19+B21</f>
-        <v>105.16</v>
+        <v>3</v>
+      </c>
+      <c r="B22" s="8">
+        <f>B20*B21</f>
+        <v>9.56</v>
       </c>
       <c r="C22" s="8"/>
-      <c r="D22" s="10">
-        <f>B22/B23</f>
-        <v>0.45119491998112154</v>
-      </c>
+      <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="8">
-        <f>B18+B22</f>
-        <v>233.07</v>
+        <v>4</v>
+      </c>
+      <c r="B23" s="14">
+        <f>B20+B22</f>
+        <v>105.16</v>
       </c>
       <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
+      <c r="D23" s="10">
+        <f>B23/B24</f>
+        <v>0.45119491998112154</v>
+      </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="8">
+        <f>B19+B23</f>
+        <v>233.07</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update decay records for 34Cl and 34S with corrections and enhancements
</commit_message>
<xml_diff>
--- a/A34/Cl34/raw/34Clm_146isomer.xlsx
+++ b/A34/Cl34/raw/34Clm_146isomer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A34\Cl34\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9FB1A2D-1EA9-4055-89ED-FA329C10806F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2197E820-FAE8-49C1-A25E-3748A8BB8F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{64E99CE1-442C-4A7F-8B3B-37F466BBE269}"/>
+    <workbookView xWindow="8004" yWindow="0" windowWidth="14508" windowHeight="12396" xr2:uid="{64E99CE1-442C-4A7F-8B3B-37F466BBE269}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -165,7 +165,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -252,6 +252,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -642,7 +645,9 @@
         <f>B3/B8</f>
         <v>0.5546023848331475</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="30">
+        <v>7.0000000000000001E-3</v>
+      </c>
       <c r="F3" s="5">
         <f>D3/B3</f>
         <v>4.2892682508364069E-3</v>
@@ -728,7 +733,9 @@
         <f>B4*B5</f>
         <v>9.4400000000000013</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2">
+        <v>0.86</v>
+      </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -754,12 +761,16 @@
         <f>B4+B6</f>
         <v>103.84</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2">
+        <v>1.8</v>
+      </c>
       <c r="D7" s="4">
         <f>B7/B8</f>
         <v>0.4453976151668525</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="E7" s="30">
+        <v>7.0000000000000001E-3</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="H7" s="22" t="s">
         <v>4</v>

</xml_diff>